<commit_message>
Commit 7 : split par type d'actifs plus portfolio  analysis
</commit_message>
<xml_diff>
--- a/Signalétique.xlsx
+++ b/Signalétique.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\seble\Code\env\Portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F38F3A-39FD-450B-99A1-D25F21A42226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D371F9-0CA7-4105-8E5C-66640C5295FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="1100" windowWidth="34590" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Positions" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="90">
   <si>
     <t>Marché</t>
   </si>
@@ -56,9 +56,6 @@
     <t>Variation %</t>
   </si>
   <si>
-    <t>AMUNDI COR STOX600</t>
-  </si>
-  <si>
     <t>MEUD</t>
   </si>
   <si>
@@ -179,15 +176,6 @@
     <t>Amundi Core Stoxx Europe 600 UCITS ETF Acc</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>Complète</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>Qualité credit</t>
   </si>
   <si>
@@ -315,6 +303,9 @@
   </si>
   <si>
     <t>CodeBank</t>
+  </si>
+  <si>
+    <t>z</t>
   </si>
 </sst>
 </file>
@@ -1290,13 +1281,13 @@
   <sheetData>
     <row r="1" spans="1:54" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -1305,290 +1296,213 @@
         <v>2</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="K1" s="2" t="s">
+      <c r="P1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="W1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AA1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="S1" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="W1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AD1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AA1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AI1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AC1" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="AK1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AE1" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AM1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="AH1" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AJ1" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="AL1" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="AO1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="AP1" s="2" t="s">
+      <c r="AT1" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="AQ1" s="2" t="s">
+      <c r="AU1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="AR1" s="2" t="s">
+      <c r="AV1" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="AS1" s="2" t="s">
+      <c r="AW1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY1" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="AT1" s="2" t="s">
+      <c r="AZ1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="BA1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="AU1" s="2" t="s">
+      <c r="BB1" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="AV1" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AW1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="AX1" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AY1" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="AZ1" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="BA1" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="BB1" s="2" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:54" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="7">
-        <v>6.9999999999999999E-4</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K2" s="7"/>
       <c r="L2" t="s">
-        <v>47</v>
-      </c>
-      <c r="N2" t="s">
-        <v>48</v>
+        <v>89</v>
       </c>
       <c r="O2">
-        <v>16513</v>
-      </c>
-      <c r="P2">
-        <v>612</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>49</v>
-      </c>
-      <c r="R2" s="8">
-        <v>0</v>
-      </c>
-      <c r="S2" s="8">
-        <v>0</v>
-      </c>
-      <c r="T2" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="U2" s="8">
-        <v>0</v>
-      </c>
-      <c r="V2" s="8">
-        <v>0</v>
-      </c>
-      <c r="W2" s="8">
-        <v>0</v>
-      </c>
-      <c r="X2" s="8">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="8">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="Z2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="8">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="AC2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AH2" s="8">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="AI2" s="8">
-        <v>0.38</v>
-      </c>
-      <c r="AJ2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AK2" s="8">
-        <v>0.18</v>
-      </c>
-      <c r="AL2" s="8">
-        <v>0.24</v>
-      </c>
-      <c r="AM2" s="8">
-        <v>0.08</v>
-      </c>
-      <c r="AN2" s="8">
-        <v>0.08</v>
-      </c>
-      <c r="AO2" s="8">
-        <v>0.11</v>
-      </c>
-      <c r="AP2" s="8">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="AQ2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AR2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AS2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AT2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AU2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AV2" s="8">
-        <v>0</v>
-      </c>
-      <c r="AW2" s="8">
-        <v>0.24</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="R2" s="8"/>
+      <c r="S2" s="8"/>
+      <c r="T2" s="8"/>
+      <c r="U2" s="8"/>
+      <c r="V2" s="8"/>
+      <c r="W2" s="8"/>
+      <c r="X2" s="8"/>
+      <c r="Y2" s="8"/>
+      <c r="Z2" s="8"/>
+      <c r="AA2" s="8"/>
+      <c r="AB2" s="8"/>
+      <c r="AC2" s="8"/>
+      <c r="AD2" s="8"/>
+      <c r="AE2" s="8"/>
+      <c r="AF2" s="8"/>
+      <c r="AG2" s="8"/>
+      <c r="AH2" s="8"/>
+      <c r="AI2" s="8"/>
+      <c r="AJ2" s="8"/>
+      <c r="AK2" s="8"/>
+      <c r="AL2" s="8"/>
+      <c r="AM2" s="8"/>
+      <c r="AN2" s="8"/>
+      <c r="AO2" s="8"/>
+      <c r="AP2" s="8"/>
+      <c r="AQ2" s="8"/>
+      <c r="AR2" s="8"/>
+      <c r="AS2" s="8"/>
+      <c r="AT2" s="8"/>
+      <c r="AU2" s="8"/>
+      <c r="AV2" s="8"/>
+      <c r="AW2" s="8"/>
       <c r="AX2" s="8"/>
       <c r="AY2" s="8"/>
       <c r="AZ2" s="8"/>
       <c r="BA2" s="8"/>
-      <c r="BB2" s="8" t="s">
-        <v>6</v>
-      </c>
+      <c r="BB2" s="8"/>
     </row>
     <row r="3" spans="1:54" x14ac:dyDescent="0.35">
       <c r="R3" s="3"/>
@@ -2542,10 +2456,10 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
         <v>8</v>
-      </c>
-      <c r="B1" t="s">
-        <v>9</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -2557,10 +2471,10 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" t="s">
         <v>10</v>
-      </c>
-      <c r="G1" t="s">
-        <v>11</v>
       </c>
       <c r="H1" t="s">
         <v>4</v>
@@ -2569,40 +2483,40 @@
         <v>5</v>
       </c>
       <c r="J1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" t="s">
         <v>12</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>13</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>14</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>15</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>16</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>17</v>
-      </c>
-      <c r="P1" t="s">
-        <v>18</v>
       </c>
       <c r="Q1" t="s">
         <v>0</v>
       </c>
       <c r="R1" t="s">
+        <v>18</v>
+      </c>
+      <c r="S1" t="s">
         <v>19</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>20</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>21</v>
-      </c>
-      <c r="U1" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -2620,30 +2534,30 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>24</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>25</v>
-      </c>
-      <c r="F1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
         <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>28</v>
       </c>
       <c r="D2" s="1">
         <v>24352.17</v>
@@ -2673,28 +2587,28 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>31</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>32</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" t="s">
         <v>33</v>
-      </c>
-      <c r="G1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I1" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>